<commit_message>
Typos and minor corrections
</commit_message>
<xml_diff>
--- a/data/percentage_rating.xlsx
+++ b/data/percentage_rating.xlsx
@@ -417,7 +417,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="str">
-        <v>97</v>
+        <v>97.5</v>
       </c>
       <c r="B2" s="1" t="str">
         <v>100</v>
@@ -431,10 +431,10 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="str">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B3" s="1" t="str">
-        <v>96</v>
+        <v>97.4</v>
       </c>
       <c r="C3" s="1" t="str">
         <v>14</v>
@@ -448,7 +448,7 @@
         <v>90</v>
       </c>
       <c r="B4" s="1" t="str">
-        <v>92</v>
+        <v>94.9</v>
       </c>
       <c r="C4" s="1" t="str">
         <v>13</v>
@@ -462,7 +462,7 @@
         <v>85</v>
       </c>
       <c r="B5" s="1" t="str">
-        <v>89</v>
+        <v>89.9</v>
       </c>
       <c r="C5" s="1" t="str">
         <v>12</v>
@@ -476,7 +476,7 @@
         <v>80</v>
       </c>
       <c r="B6" s="1" t="str">
-        <v>84</v>
+        <v>84.9</v>
       </c>
       <c r="C6" s="1" t="str">
         <v>11</v>
@@ -490,7 +490,7 @@
         <v>75</v>
       </c>
       <c r="B7" s="1" t="str">
-        <v>79</v>
+        <v>79.9</v>
       </c>
       <c r="C7" s="1" t="str">
         <v>10</v>
@@ -504,7 +504,7 @@
         <v>70</v>
       </c>
       <c r="B8" s="1" t="str">
-        <v>74</v>
+        <v>74.9</v>
       </c>
       <c r="C8" s="1" t="str">
         <v>9</v>
@@ -518,7 +518,7 @@
         <v>65</v>
       </c>
       <c r="B9" s="1" t="str">
-        <v>69</v>
+        <v>69.9</v>
       </c>
       <c r="C9" s="1" t="str">
         <v>8</v>
@@ -532,7 +532,7 @@
         <v>60</v>
       </c>
       <c r="B10" s="1" t="str">
-        <v>64</v>
+        <v>64.9</v>
       </c>
       <c r="C10" s="1" t="str">
         <v>7</v>
@@ -546,7 +546,7 @@
         <v>55</v>
       </c>
       <c r="B11" s="1" t="str">
-        <v>59</v>
+        <v>59.9</v>
       </c>
       <c r="C11" s="1" t="str">
         <v>6</v>
@@ -560,7 +560,7 @@
         <v>50</v>
       </c>
       <c r="B12" s="1" t="str">
-        <v>54</v>
+        <v>54.9</v>
       </c>
       <c r="C12" s="1" t="str">
         <v>5</v>
@@ -574,7 +574,7 @@
         <v>45</v>
       </c>
       <c r="B13" s="1" t="str">
-        <v>49</v>
+        <v>49.9</v>
       </c>
       <c r="C13" s="1" t="str">
         <v>4</v>
@@ -585,10 +585,10 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="str">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B14" s="1" t="str">
-        <v>44</v>
+        <v>44.9</v>
       </c>
       <c r="C14" s="1" t="str">
         <v>3</v>
@@ -599,10 +599,10 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="str">
-        <v>32</v>
+        <v>32.5</v>
       </c>
       <c r="B15" s="1" t="str">
-        <v>37</v>
+        <v>39.9</v>
       </c>
       <c r="C15" s="1" t="str">
         <v>2</v>
@@ -616,7 +616,7 @@
         <v>25</v>
       </c>
       <c r="B16" s="1" t="str">
-        <v>31</v>
+        <v>32.4</v>
       </c>
       <c r="C16" s="1" t="str">
         <v>1</v>
@@ -630,7 +630,7 @@
         <v>0</v>
       </c>
       <c r="B17" s="1" t="str">
-        <v>25</v>
+        <v>24.9</v>
       </c>
       <c r="C17" s="1" t="str">
         <v>0</v>

</xml_diff>